<commit_message>
ring: training-data paper also under Research Practice; news: post about the site redesign
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/areas.xlsx
+++ b/data/areas.xlsx
@@ -1568,7 +1568,11 @@
           <t>Nonverbal Behavior</t>
         </is>
       </c>
-      <c r="H25" s="3" t="n"/>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Research Practice</t>
+        </is>
+      </c>
       <c r="I25" s="6" t="n"/>
       <c r="J25" s="2" t="n"/>
     </row>
@@ -3511,7 +3515,7 @@
   </sheetData>
   <autoFilter ref="A1:J72"/>
   <dataValidations count="1">
-    <dataValidation sqref="F2:I72" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an area" error="Pick a subarea from the Areas sheet, or leave blank." type="list">
+    <dataValidation sqref="F2:I72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Areas!$B$2:$B$11</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
publications: Kebe et al. 2026 TACL paper (LlaMADRS); ring and pubs data rebuilt
</commit_message>
<xml_diff>
--- a/data/areas.xlsx
+++ b/data/areas.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Areas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Papers" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Questions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Areas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="How to use" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Papers'!$A$1:$J$72</definedName>
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2523,22 +2523,22 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>kim2023</t>
+          <t>kebe2026</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Human and Machine Recognition of Dynamic and Static Facial Expressions: Prototypicality, Ambiguity, and Complexity</t>
+          <t>LlaMADRS: Evaluating Open-Source LLMs on Real Clinical Interviews—To Reason or Not to Reason?</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Frontiers in Psychology</t>
+          <t>Transactions of the Association for Computational Linguistics</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -2548,17 +2548,17 @@
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>Nonverbal Behavior</t>
+          <t>Artificial Intelligence</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>Social Perception</t>
+          <t>Clinical Assessment</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>Artificial Intelligence</t>
+          <t>Verbal Behavior</t>
         </is>
       </c>
       <c r="I49" s="6" t="n"/>
@@ -2567,22 +2567,22 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>lin2020</t>
+          <t>kim2023</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Toward Multimodal Modeling of Emotional Expressiveness</t>
+          <t>Human and Machine Recognition of Dynamic and Static Facial Expressions: Prototypicality, Ambiguity, and Complexity</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Proceedings of the 22nd International Conference on Multimodal Interaction</t>
+          <t>Frontiers in Psychology</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2592,17 +2592,17 @@
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
+          <t>Nonverbal Behavior</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Social Perception</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
           <t>Artificial Intelligence</t>
-        </is>
-      </c>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>Nonverbal Behavior</t>
-        </is>
-      </c>
-      <c r="H50" s="3" t="inlineStr">
-        <is>
-          <t>Social Perception</t>
         </is>
       </c>
       <c r="I50" s="6" t="n"/>
@@ -2611,7 +2611,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>lin2020a</t>
+          <t>lin2020</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2621,12 +2621,12 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Context-Dependent Models for Predicting and Characterizing Facial Expressiveness</t>
+          <t>Toward Multimodal Modeling of Emotional Expressiveness</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Proceedings of the 3rd Workshop on Affective Content Analysis Co-Located with the 34th AAAI Conference on Artificial Intelligence</t>
+          <t>Proceedings of the 22nd International Conference on Multimodal Interaction</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -2655,22 +2655,22 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>linsalata2024</t>
+          <t>lin2020a</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Sources of Environmental Reinforcement and Engagement in Health Risk Behaviors among a General Population Sample of US Adults</t>
+          <t>Context-Dependent Models for Predicting and Characterizing Facial Expressiveness</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>International Journal of Environmental Research and Public Health</t>
+          <t>Proceedings of the 3rd Workshop on Affective Content Analysis Co-Located with the 34th AAAI Conference on Artificial Intelligence</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2680,37 +2680,41 @@
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Clinical Mechanisms</t>
+          <t>Artificial Intelligence</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>Statistical Modeling</t>
-        </is>
-      </c>
-      <c r="H52" s="3" t="n"/>
+          <t>Nonverbal Behavior</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>Social Perception</t>
+        </is>
+      </c>
       <c r="I52" s="6" t="n"/>
       <c r="J52" s="2" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>mcduff2017</t>
+          <t>linsalata2024</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Large-Scale Observational Evidence of Cross-Cultural Differences in Facial Behavior</t>
+          <t>Sources of Environmental Reinforcement and Engagement in Health Risk Behaviors among a General Population Sample of US Adults</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Journal of Nonverbal Behavior</t>
+          <t>International Journal of Environmental Research and Public Health</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -2720,12 +2724,12 @@
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>Nonverbal Behavior</t>
+          <t>Clinical Mechanisms</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>Artificial Intelligence</t>
+          <t>Statistical Modeling</t>
         </is>
       </c>
       <c r="H53" s="3" t="n"/>
@@ -2735,22 +2739,22 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>mcduff2019</t>
+          <t>mcduff2017</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2017</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Democratizing Psychological Insights from Analysis of Nonverbal Behavior</t>
+          <t>Large-Scale Observational Evidence of Cross-Cultural Differences in Facial Behavior</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Proceedings of the 8th International Conference on Affective Computing and Intelligent Interaction (ACII)</t>
+          <t>Journal of Nonverbal Behavior</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -2775,22 +2779,22 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>muszynski2020</t>
+          <t>mcduff2019</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Depression Severity Assessment for Adolescents at High Risk of Mental Disorders</t>
+          <t>Democratizing Psychological Insights from Analysis of Nonverbal Behavior</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Proceedings of the 22nd International Conference on Multimodal Interaction</t>
+          <t>Proceedings of the 8th International Conference on Affective Computing and Intelligent Interaction (ACII)</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -2800,12 +2804,12 @@
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
+          <t>Nonverbal Behavior</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
           <t>Artificial Intelligence</t>
-        </is>
-      </c>
-      <c r="G55" s="3" t="inlineStr">
-        <is>
-          <t>Clinical Assessment</t>
         </is>
       </c>
       <c r="H55" s="3" t="n"/>
@@ -2815,22 +2819,22 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>pacella2018</t>
+          <t>muszynski2020</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>The Association between Daily Posttraumatic Stress Symptoms and Pain over the First 14 Days after Injury: An Experience Sampling Study</t>
+          <t>Depression Severity Assessment for Adolescents at High Risk of Mental Disorders</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Academic Emergency Medicine</t>
+          <t>Proceedings of the 22nd International Conference on Multimodal Interaction</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -2840,12 +2844,12 @@
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>Clinical Mechanisms</t>
+          <t>Artificial Intelligence</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>Statistical Modeling</t>
+          <t>Clinical Assessment</t>
         </is>
       </c>
       <c r="H56" s="3" t="n"/>
@@ -2855,22 +2859,22 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>rinconcaicedo2025</t>
+          <t>pacella2018</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Depressive Symptoms among Hispanic Americans: Investigating the Interplay of Acculturation and Demographics</t>
+          <t>The Association between Daily Posttraumatic Stress Symptoms and Pain over the First 14 Days after Injury: An Experience Sampling Study</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Journal of Latinx Psychology</t>
+          <t>Academic Emergency Medicine</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -2895,22 +2899,22 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>ross2017</t>
+          <t>rinconcaicedo2025</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Momentary Patterns of Covariation between Specific Affects and Interpersonal Behavior: Linking Relationship Science and Personality Assessment</t>
+          <t>Depressive Symptoms among Hispanic Americans: Investigating the Interplay of Acculturation and Demographics</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Psychological Assessment</t>
+          <t>Journal of Latinx Psychology</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -2920,7 +2924,7 @@
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>Interpersonal Dynamics</t>
+          <t>Clinical Mechanisms</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
@@ -2928,33 +2932,29 @@
           <t>Statistical Modeling</t>
         </is>
       </c>
-      <c r="H58" s="3" t="inlineStr">
-        <is>
-          <t>Nonverbal Behavior</t>
-        </is>
-      </c>
+      <c r="H58" s="3" t="n"/>
       <c r="I58" s="6" t="n"/>
       <c r="J58" s="2" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>setiawan2025</t>
+          <t>ross2017</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2017</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Individualized Machine-Learning-Based Clinical Assessment Recommendation System</t>
+          <t>Momentary Patterns of Covariation between Specific Affects and Interpersonal Behavior: Linking Relationship Science and Personality Assessment</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>PLOS Digital Health</t>
+          <t>Psychological Assessment</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -2964,37 +2964,41 @@
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>Artificial Intelligence</t>
+          <t>Interpersonal Dynamics</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>Clinical Assessment</t>
-        </is>
-      </c>
-      <c r="H59" s="3" t="n"/>
+          <t>Statistical Modeling</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>Nonverbal Behavior</t>
+        </is>
+      </c>
       <c r="I59" s="6" t="n"/>
       <c r="J59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>sewall2021</t>
+          <t>setiawan2025</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>A Bayesian Multilevel Analysis of the Longitudinal Associations between Relationship Quality and Suicidal Ideation and Attempts among Youth with Bipolar Disorder</t>
+          <t>Individualized Machine-Learning-Based Clinical Assessment Recommendation System</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>The Journal of Child Psychology and Psychiatry</t>
+          <t>PLOS Digital Health</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -3004,41 +3008,37 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Clinical Mechanisms</t>
+          <t>Artificial Intelligence</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>Statistical Modeling</t>
-        </is>
-      </c>
-      <c r="H60" s="3" t="inlineStr">
-        <is>
-          <t>Interpersonal Dynamics</t>
-        </is>
-      </c>
+          <t>Clinical Assessment</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="n"/>
       <c r="I60" s="6" t="n"/>
       <c r="J60" s="2" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>shepherd2017</t>
+          <t>sewall2021</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Comparison of Comprehensive and Abstinence-Only Sexuality Education in Young African American Adolescents</t>
+          <t>A Bayesian Multilevel Analysis of the Longitudinal Associations between Relationship Quality and Suicidal Ideation and Attempts among Youth with Bipolar Disorder</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Journal of Adolescence</t>
+          <t>The Journal of Child Psychology and Psychiatry</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -3046,48 +3046,52 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F61" s="3" t="n"/>
-      <c r="G61" s="3" t="n"/>
-      <c r="H61" s="3" t="n"/>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>Clinical Mechanisms</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>Statistical Modeling</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>Interpersonal Dynamics</t>
+        </is>
+      </c>
       <c r="I61" s="6" t="n"/>
       <c r="J61" s="2" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>sprunger2024</t>
+          <t>shepherd2017</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2017</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Associations between Transdiagnostic Traits of Psychopathology and Hybrid Posttraumatic Stress Disorder Factors in a Trauma-Exposed Community Sample</t>
+          <t>Comparison of Comprehensive and Abstinence-Only Sexuality Education in Young African American Adolescents</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Journal of Traumatic Stress</t>
+          <t>Journal of Adolescence</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F62" s="3" t="inlineStr">
-        <is>
-          <t>Clinical Assessment</t>
-        </is>
-      </c>
-      <c r="G62" s="3" t="inlineStr">
-        <is>
-          <t>Statistical Modeling</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="n"/>
+      <c r="G62" s="3" t="n"/>
       <c r="H62" s="3" t="n"/>
       <c r="I62" s="6" t="n"/>
       <c r="J62" s="2" t="n"/>
@@ -3095,35 +3099,39 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>swartz2023</t>
+          <t>sprunger2024</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Randomized Trial of Brief Interpersonal Psychotherapy and Cognitive Behavioral Therapy for Depression Delivered Both In-Person and by Telehealth</t>
+          <t>Associations between Transdiagnostic Traits of Psychopathology and Hybrid Posttraumatic Stress Disorder Factors in a Trauma-Exposed Community Sample</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Journal of Affective Disorders</t>
+          <t>Journal of Traumatic Stress</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Clinical Mechanisms</t>
-        </is>
-      </c>
-      <c r="G63" s="3" t="n"/>
+          <t>Clinical Assessment</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>Statistical Modeling</t>
+        </is>
+      </c>
       <c r="H63" s="3" t="n"/>
       <c r="I63" s="6" t="n"/>
       <c r="J63" s="2" t="n"/>
@@ -3131,22 +3139,22 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>vail2021</t>
+          <t>swartz2023</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Goals, Tasks, and Bonds: Toward the Computational Assessment of Therapist versus Client Perception of Working Alliance</t>
+          <t>Randomized Trial of Brief Interpersonal Psychotherapy and Cognitive Behavioral Therapy for Depression Delivered Both In-Person and by Telehealth</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Proceedings of the 16th IEEE International Conference on Automatic Face and Gesture Recognition (FG)</t>
+          <t>Journal of Affective Disorders</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -3159,38 +3167,30 @@
           <t>Clinical Mechanisms</t>
         </is>
       </c>
-      <c r="G64" s="3" t="inlineStr">
-        <is>
-          <t>Artificial Intelligence</t>
-        </is>
-      </c>
-      <c r="H64" s="3" t="inlineStr">
-        <is>
-          <t>Interpersonal Dynamics</t>
-        </is>
-      </c>
+      <c r="G64" s="3" t="n"/>
+      <c r="H64" s="3" t="n"/>
       <c r="I64" s="6" t="n"/>
       <c r="J64" s="2" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>vail2022</t>
+          <t>vail2021</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Toward Causal Understanding of Therapist-Client Relationships: A Study of Language Modality and Social Entrainment</t>
+          <t>Goals, Tasks, and Bonds: Toward the Computational Assessment of Therapist versus Client Perception of Working Alliance</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Proceedings of the 24th ACM International Conference on Multimodal Interaction</t>
+          <t>Proceedings of the 16th IEEE International Conference on Automatic Face and Gesture Recognition (FG)</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -3205,12 +3205,12 @@
       </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
           <t>Interpersonal Dynamics</t>
-        </is>
-      </c>
-      <c r="H65" s="3" t="inlineStr">
-        <is>
-          <t>Verbal Behavior</t>
         </is>
       </c>
       <c r="I65" s="6" t="n"/>
@@ -3219,22 +3219,22 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>vail2023</t>
+          <t>vail2022</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Representation Learning for Interpersonal and Multimodal Behavior Dynamics: A Multiview Extension of Latent Change Score Models</t>
+          <t>Toward Causal Understanding of Therapist-Client Relationships: A Study of Language Modality and Social Entrainment</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Proceedings of the 25th International Conference on Multimodal Interaction</t>
+          <t>Proceedings of the 24th ACM International Conference on Multimodal Interaction</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -3244,17 +3244,17 @@
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Artificial Intelligence</t>
+          <t>Clinical Mechanisms</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
         <is>
-          <t>Statistical Modeling</t>
+          <t>Interpersonal Dynamics</t>
         </is>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>Interpersonal Dynamics</t>
+          <t>Verbal Behavior</t>
         </is>
       </c>
       <c r="I66" s="6" t="n"/>
@@ -3263,22 +3263,22 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>valstar2015</t>
+          <t>vail2023</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>FERA 2015 - Second Facial Expression Recognition and Analysis Challenge</t>
+          <t>Representation Learning for Interpersonal and Multimodal Behavior Dynamics: A Multiview Extension of Latent Change Score Models</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Proceedings of the 11th IEEE International Conference on Automatic Face and Gesture Recognition (FG)</t>
+          <t>Proceedings of the 25th International Conference on Multimodal Interaction</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -3288,17 +3288,17 @@
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Open Resources</t>
+          <t>Artificial Intelligence</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
         <is>
-          <t>Artificial Intelligence</t>
+          <t>Statistical Modeling</t>
         </is>
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>Nonverbal Behavior</t>
+          <t>Interpersonal Dynamics</t>
         </is>
       </c>
       <c r="I67" s="6" t="n"/>
@@ -3307,22 +3307,22 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>valstar2017</t>
+          <t>valstar2015</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2015</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>FERA 2017 - Addressing Head Pose in the Third Facial Expression Recognition and Analysis Challenge</t>
+          <t>FERA 2015 - Second Facial Expression Recognition and Analysis Challenge</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Proceedings of the 12th IEEE Conference on Automatic Face and Gesture Recognition (FG)</t>
+          <t>Proceedings of the 11th IEEE International Conference on Automatic Face and Gesture Recognition (FG)</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -3351,22 +3351,22 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>vanoest2022</t>
+          <t>valstar2017</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2017</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Weighting Schemes and Incomplete Data: A Generalized Bayesian Framework for Chance-Corrected Interrater Agreement</t>
+          <t>FERA 2017 - Addressing Head Pose in the Third Facial Expression Recognition and Analysis Challenge</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Psychological Methods</t>
+          <t>Proceedings of the 12th IEEE Conference on Automatic Face and Gesture Recognition (FG)</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -3376,37 +3376,41 @@
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Statistical Modeling</t>
+          <t>Open Resources</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
         <is>
-          <t>Research Practice</t>
-        </is>
-      </c>
-      <c r="H69" s="3" t="n"/>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>Nonverbal Behavior</t>
+        </is>
+      </c>
       <c r="I69" s="6" t="n"/>
       <c r="J69" s="2" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>wolfert2021</t>
+          <t>vanoest2022</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>To Rate or Not to Rate: Investigating Evaluation Methods for Generated Co-Speech Gestures</t>
+          <t>Weighting Schemes and Incomplete Data: A Generalized Bayesian Framework for Chance-Corrected Interrater Agreement</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Proceedings of the 23rd International Conference on Multimodal Interaction</t>
+          <t>Psychological Methods</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -3416,41 +3420,37 @@
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
+          <t>Statistical Modeling</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
           <t>Research Practice</t>
         </is>
       </c>
-      <c r="G70" s="3" t="inlineStr">
-        <is>
-          <t>Artificial Intelligence</t>
-        </is>
-      </c>
-      <c r="H70" s="3" t="inlineStr">
-        <is>
-          <t>Nonverbal Behavior</t>
-        </is>
-      </c>
+      <c r="H70" s="3" t="n"/>
       <c r="I70" s="6" t="n"/>
       <c r="J70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>zhang2014</t>
+          <t>wolfert2021</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>BP4D-spontaneous: A High-Resolution Spontaneous 3D Dynamic Facial Expression Database</t>
+          <t>To Rate or Not to Rate: Investigating Evaluation Methods for Generated Co-Speech Gestures</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Image and Vision Computing</t>
+          <t>Proceedings of the 23rd International Conference on Multimodal Interaction</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -3460,37 +3460,41 @@
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Open Resources</t>
+          <t>Research Practice</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
           <t>Nonverbal Behavior</t>
         </is>
       </c>
-      <c r="H71" s="3" t="n"/>
       <c r="I71" s="6" t="n"/>
       <c r="J71" s="2" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>zhang2016</t>
+          <t>zhang2014</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Multimodal Spontaneous Emotion Corpus for Human Behavior Analysis</t>
+          <t>BP4D-spontaneous: A High-Resolution Spontaneous 3D Dynamic Facial Expression Database</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Proceedings of the IEEE Conference on Computer Vision and Pattern Recognition (CVPR)</t>
+          <t>Image and Vision Computing</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -3511,6 +3515,46 @@
       <c r="H72" s="3" t="n"/>
       <c r="I72" s="6" t="n"/>
       <c r="J72" s="2" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>zhang2016</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Multimodal Spontaneous Emotion Corpus for Human Behavior Analysis</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Proceedings of the IEEE Conference on Computer Vision and Pattern Recognition (CVPR)</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>Open Resources</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>Nonverbal Behavior</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="n"/>
+      <c r="I73" s="6" t="n"/>
+      <c r="J73" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J72"/>

</xml_diff>